<commit_message>
added transport and catering fee to view info page, added header to ticket csv file, changed usernames
</commit_message>
<xml_diff>
--- a/database/users.xlsx
+++ b/database/users.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Username</t>
   </si>
@@ -25,13 +25,19 @@
     <t>Role</t>
   </si>
   <si>
-    <t>abc</t>
+    <t>STU1</t>
   </si>
   <si>
     <t>STUDENT</t>
   </si>
   <si>
+    <t>EO1</t>
+  </si>
+  <si>
     <t>EO</t>
+  </si>
+  <si>
+    <t>STA1</t>
   </si>
   <si>
     <t>STAFF</t>
@@ -90,18 +96,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -416,11 +425,11 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -435,33 +444,33 @@
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="2">
         <v>123</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="2" t="s">
-        <v>3</v>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+      <c r="A3" s="4" t="s">
+        <v>5</v>
       </c>
       <c r="B3" s="2">
         <v>456</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="4">
+      <c r="A4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2">
         <v>789</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>